<commit_message>
Updated daily Excel details
</commit_message>
<xml_diff>
--- a/12628332.xlsx
+++ b/12628332.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cap776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27A1E6DF-559C-4D76-9571-CC5DBA5124DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B455133F-996E-4157-A702-CE0B0AFBB1E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="77">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -211,9 +211,6 @@
     <t>MCA</t>
   </si>
   <si>
-    <t>28/08/2026</t>
-  </si>
-  <si>
     <t>feeling is not so great</t>
   </si>
   <si>
@@ -221,9 +218,6 @@
   </si>
   <si>
     <t>Low</t>
-  </si>
-  <si>
-    <t>29/08/2026</t>
   </si>
   <si>
     <t>Excellent</t>
@@ -235,13 +229,7 @@
     <t>this day was very good</t>
   </si>
   <si>
-    <t>30/08/2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">it was a nice day </t>
-  </si>
-  <si>
-    <t>31/08/2026</t>
   </si>
   <si>
     <t>this was just a normal day</t>
@@ -251,6 +239,33 @@
   </si>
   <si>
     <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>2026/31/08</t>
+  </si>
+  <si>
+    <t>2026/30/08</t>
+  </si>
+  <si>
+    <t>2026/29/08</t>
+  </si>
+  <si>
+    <t>2026/28/08</t>
+  </si>
+  <si>
+    <t>good</t>
+  </si>
+  <si>
+    <t xml:space="preserve">just average </t>
+  </si>
+  <si>
+    <t xml:space="preserve">average </t>
+  </si>
+  <si>
+    <t>satisfied</t>
+  </si>
+  <si>
+    <t>high</t>
   </si>
 </sst>
 </file>
@@ -1082,7 +1097,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="B7" s="14">
         <v>450</v>
@@ -1114,21 +1129,21 @@
         <v>500</v>
       </c>
       <c r="K7" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L7" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M7" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="L7" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="M7" s="16" t="s">
-        <v>61</v>
-      </c>
       <c r="N7" s="17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="B8" s="14">
         <v>500</v>
@@ -1160,21 +1175,21 @@
         <v>260</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L8" s="16" t="s">
         <v>50</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="N8" s="17" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B9" s="14">
         <v>500</v>
@@ -1206,16 +1221,16 @@
         <v>320</v>
       </c>
       <c r="K9" s="16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L9" s="16" t="s">
         <v>50</v>
       </c>
       <c r="M9" s="16" t="s">
+        <v>62</v>
+      </c>
+      <c r="N9" s="17" t="s">
         <v>64</v>
-      </c>
-      <c r="N9" s="17" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
@@ -1255,13 +1270,13 @@
         <v>49</v>
       </c>
       <c r="L10" s="16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M10" s="16" t="s">
         <v>51</v>
       </c>
       <c r="N10" s="17" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
@@ -1307,12 +1322,12 @@
         <v>51</v>
       </c>
       <c r="N11" s="17" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="13">
-        <v>46031</v>
+        <v>46062</v>
       </c>
       <c r="B12" s="14">
         <v>480</v>
@@ -1344,61 +1359,109 @@
         <v>150</v>
       </c>
       <c r="K12" s="16" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L12" s="16" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="M12" s="16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="N12" s="17" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="13"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15" t="str">
+      <c r="A13" s="13">
+        <v>46090</v>
+      </c>
+      <c r="B13" s="14">
+        <v>500</v>
+      </c>
+      <c r="C13" s="14">
+        <v>30</v>
+      </c>
+      <c r="D13" s="14">
+        <v>200</v>
+      </c>
+      <c r="E13" s="14">
+        <v>50</v>
+      </c>
+      <c r="F13" s="14">
+        <v>300</v>
+      </c>
+      <c r="G13" s="14">
+        <v>6</v>
+      </c>
+      <c r="H13" s="14">
+        <v>200</v>
+      </c>
+      <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" s="15" t="str">
+        <v>1280</v>
+      </c>
+      <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="17"/>
+        <v>160</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N13" s="17" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15" t="str">
+      <c r="A14" s="13">
+        <v>46121</v>
+      </c>
+      <c r="B14" s="14">
+        <v>400</v>
+      </c>
+      <c r="C14" s="14">
+        <v>50</v>
+      </c>
+      <c r="D14" s="14">
+        <v>150</v>
+      </c>
+      <c r="E14" s="14">
+        <v>150</v>
+      </c>
+      <c r="F14" s="14">
+        <v>250</v>
+      </c>
+      <c r="G14" s="14">
+        <v>5</v>
+      </c>
+      <c r="H14" s="14">
+        <v>160</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+        <v>1160</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="17"/>
+        <v>280</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="13"/>

</xml_diff>